<commit_message>
Update Faixa Etaria e Ticket data
</commit_message>
<xml_diff>
--- a/Arquivos Jun-2026/Compra x Recência x Ticket Médio.xlsx
+++ b/Arquivos Jun-2026/Compra x Recência x Ticket Médio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://farmaciassaojoao-my.sharepoint.com/personal/chaiani_savedra_farmaciassaojoao_com_br/Documents/Área de Trabalho/Antigravity/CRM - V4/Arquivos Jun-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{37F5FAB6-688A-41F4-B6E2-5823BB444B99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E70E70D9-791B-4524-964E-EB0AFBF04CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{A1F6043E-F109-48E6-886C-BB2489C13DFF}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{185380D6-F1C4-46D0-AAC3-9C8E9B59E74F}"/>
   </bookViews>
   <sheets>
     <sheet name="Frequência × Recência × ticket " sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="116">
   <si>
     <t>FAIXA_RECENCIA</t>
   </si>
@@ -46,28 +46,28 @@
     <t>PCT_FATURAMENTO</t>
   </si>
   <si>
-    <t>693842802.81</t>
-  </si>
-  <si>
-    <t>81.09</t>
-  </si>
-  <si>
-    <t>0.45</t>
+    <t>694509050.95</t>
+  </si>
+  <si>
+    <t>81.1</t>
+  </si>
+  <si>
+    <t>0.46</t>
   </si>
   <si>
     <t>12.86</t>
   </si>
   <si>
-    <t>5 - Até 30 dias</t>
-  </si>
-  <si>
-    <t>1 - Até 1 transação</t>
-  </si>
-  <si>
-    <t>20392680.14</t>
-  </si>
-  <si>
-    <t>83.27</t>
+    <t>5 - AtÃ© 30 dias</t>
+  </si>
+  <si>
+    <t>1 - AtÃ© 1 transaÃ§Ã£o</t>
+  </si>
+  <si>
+    <t>20416382.87</t>
+  </si>
+  <si>
+    <t>83.25</t>
   </si>
   <si>
     <t>2.73</t>
@@ -76,13 +76,13 @@
     <t>0.38</t>
   </si>
   <si>
-    <t>2 - Entre 2 e 3 transações</t>
-  </si>
-  <si>
-    <t>67138566.36</t>
-  </si>
-  <si>
-    <t>78.68</t>
+    <t>2 - Entre 2 e 3 transaÃ§Ãµes</t>
+  </si>
+  <si>
+    <t>67218041.27</t>
+  </si>
+  <si>
+    <t>78.69</t>
   </si>
   <si>
     <t>4.89</t>
@@ -91,10 +91,10 @@
     <t>1.24</t>
   </si>
   <si>
-    <t>3 - Entre 4 e 6 transações</t>
-  </si>
-  <si>
-    <t>157072210.16</t>
+    <t>3 - Entre 4 e 6 transaÃ§Ãµes</t>
+  </si>
+  <si>
+    <t>157227355.71</t>
   </si>
   <si>
     <t>79.1</t>
@@ -106,10 +106,10 @@
     <t>2.91</t>
   </si>
   <si>
-    <t>4 - Entre 7 e 13 transações</t>
-  </si>
-  <si>
-    <t>542819188.62</t>
+    <t>4 - Entre 7 e 13 transaÃ§Ãµes</t>
+  </si>
+  <si>
+    <t>543306016.1</t>
   </si>
   <si>
     <t>81.61</t>
@@ -121,28 +121,28 @@
     <t>10.06</t>
   </si>
   <si>
-    <t>5 - Acima de 14 transações</t>
-  </si>
-  <si>
-    <t>2906468545.99</t>
+    <t>5 - Acima de 14 transaÃ§Ãµes</t>
+  </si>
+  <si>
+    <t>2909024936.74</t>
   </si>
   <si>
     <t>86.87</t>
   </si>
   <si>
-    <t>22.57</t>
-  </si>
-  <si>
-    <t>53.86</t>
+    <t>22.56</t>
+  </si>
+  <si>
+    <t>53.85</t>
   </si>
   <si>
     <t>4 - Entre 31 e 60 dias</t>
   </si>
   <si>
-    <t>17440080.34</t>
-  </si>
-  <si>
-    <t>76.47</t>
+    <t>17459178.91</t>
+  </si>
+  <si>
+    <t>76.48</t>
   </si>
   <si>
     <t>2.54</t>
@@ -151,7 +151,7 @@
     <t>0.32</t>
   </si>
   <si>
-    <t>48713219.53</t>
+    <t>48752947.23</t>
   </si>
   <si>
     <t>76.26</t>
@@ -163,10 +163,7 @@
     <t>0.9</t>
   </si>
   <si>
-    <t>88261560.99</t>
-  </si>
-  <si>
-    <t>77.06</t>
+    <t>77.07</t>
   </si>
   <si>
     <t>4.17</t>
@@ -175,10 +172,10 @@
     <t>1.64</t>
   </si>
   <si>
-    <t>187314429.35</t>
-  </si>
-  <si>
-    <t>79.04</t>
+    <t>187493374.11</t>
+  </si>
+  <si>
+    <t>79.05</t>
   </si>
   <si>
     <t>5.08</t>
@@ -187,10 +184,10 @@
     <t>3.47</t>
   </si>
   <si>
-    <t>208782567.1</t>
-  </si>
-  <si>
-    <t>79.67</t>
+    <t>208996533.76</t>
+  </si>
+  <si>
+    <t>79.68</t>
   </si>
   <si>
     <t>2.82</t>
@@ -202,10 +199,7 @@
     <t>3 - Entre 61 e 90 dias</t>
   </si>
   <si>
-    <t>16092756.83</t>
-  </si>
-  <si>
-    <t>79.02</t>
+    <t>16108889.58</t>
   </si>
   <si>
     <t>2.27</t>
@@ -214,10 +208,10 @@
     <t>0.3</t>
   </si>
   <si>
-    <t>35697771.96</t>
-  </si>
-  <si>
-    <t>75.48</t>
+    <t>35726169.3</t>
+  </si>
+  <si>
+    <t>75.49</t>
   </si>
   <si>
     <t>3.06</t>
@@ -226,7 +220,7 @@
     <t>0.66</t>
   </si>
   <si>
-    <t>50661296.84</t>
+    <t>50702851.27</t>
   </si>
   <si>
     <t>76.94</t>
@@ -238,10 +232,10 @@
     <t>0.94</t>
   </si>
   <si>
-    <t>70411609.63</t>
-  </si>
-  <si>
-    <t>78.22</t>
+    <t>70476913.1</t>
+  </si>
+  <si>
+    <t>78.23</t>
   </si>
   <si>
     <t>2.23</t>
@@ -250,10 +244,10 @@
     <t>1.3</t>
   </si>
   <si>
-    <t>37552251.9</t>
-  </si>
-  <si>
-    <t>74.25</t>
+    <t>37580363.3</t>
+  </si>
+  <si>
+    <t>74.26</t>
   </si>
   <si>
     <t>0.65</t>
@@ -265,7 +259,7 @@
     <t>2 - Entre 91 e 180 dias</t>
   </si>
   <si>
-    <t>45752151.83</t>
+    <t>45777625.24</t>
   </si>
   <si>
     <t>78.98</t>
@@ -277,7 +271,7 @@
     <t>0.85</t>
   </si>
   <si>
-    <t>67609786.35</t>
+    <t>67656590.45</t>
   </si>
   <si>
     <t>75.8</t>
@@ -289,7 +283,7 @@
     <t>1.25</t>
   </si>
   <si>
-    <t>59135877.13</t>
+    <t>59182833.25</t>
   </si>
   <si>
     <t>76.95</t>
@@ -301,7 +295,7 @@
     <t>1.1</t>
   </si>
   <si>
-    <t>46310293.17</t>
+    <t>46346141.23</t>
   </si>
   <si>
     <t>77.7</t>
@@ -313,7 +307,7 @@
     <t>0.86</t>
   </si>
   <si>
-    <t>16024614.04</t>
+    <t>16032888.85</t>
   </si>
   <si>
     <t>71.56</t>
@@ -325,10 +319,10 @@
     <t>1 - Acima de 181 dias</t>
   </si>
   <si>
-    <t>5735442.67</t>
-  </si>
-  <si>
-    <t>80.42</t>
+    <t>5773493.88</t>
+  </si>
+  <si>
+    <t>80.36</t>
   </si>
   <si>
     <t>0.80</t>
@@ -337,10 +331,7 @@
     <t>0.11</t>
   </si>
   <si>
-    <t>4885070.74</t>
-  </si>
-  <si>
-    <t>79.01</t>
+    <t>4916952.42</t>
   </si>
   <si>
     <t>0.60</t>
@@ -349,34 +340,34 @@
     <t>0.09</t>
   </si>
   <si>
-    <t>1980184.35</t>
-  </si>
-  <si>
-    <t>80.27</t>
-  </si>
-  <si>
-    <t>0.22</t>
+    <t>1989749.46</t>
+  </si>
+  <si>
+    <t>80.21</t>
+  </si>
+  <si>
+    <t>0.23</t>
   </si>
   <si>
     <t>0.04</t>
   </si>
   <si>
-    <t>604804.71</t>
+    <t>607541.32</t>
   </si>
   <si>
     <t>79.09</t>
   </si>
   <si>
-    <t>0.06</t>
+    <t>0.07</t>
   </si>
   <si>
     <t>0.01</t>
   </si>
   <si>
-    <t>99996.2</t>
-  </si>
-  <si>
-    <t>72.94</t>
+    <t>100045.59</t>
+  </si>
+  <si>
+    <t>72.87</t>
   </si>
 </sst>
 </file>
@@ -1236,13 +1227,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8B7EAA3-AB1E-4CFB-850B-AEB282ACB203}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E49846D-C7B6-4C24-947E-14692BBDA877}">
   <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="1" max="1" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1273,10 +1262,10 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C2">
-        <v>40029</v>
+        <v>41009</v>
       </c>
       <c r="D2">
-        <v>8556651</v>
+        <v>8563198</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -1302,7 +1291,7 @@
         <v>243979</v>
       </c>
       <c r="D3">
-        <v>244894</v>
+        <v>245234</v>
       </c>
       <c r="E3" t="s">
         <v>14</v>
@@ -1328,7 +1317,7 @@
         <v>437799</v>
       </c>
       <c r="D4">
-        <v>853264</v>
+        <v>854239</v>
       </c>
       <c r="E4" t="s">
         <v>19</v>
@@ -1354,7 +1343,7 @@
         <v>584290</v>
       </c>
       <c r="D5">
-        <v>1985809</v>
+        <v>1987820</v>
       </c>
       <c r="E5" t="s">
         <v>24</v>
@@ -1380,7 +1369,7 @@
         <v>1097136</v>
       </c>
       <c r="D6">
-        <v>6651517</v>
+        <v>6657577</v>
       </c>
       <c r="E6" t="s">
         <v>29</v>
@@ -1406,7 +1395,7 @@
         <v>2018621</v>
       </c>
       <c r="D7">
-        <v>33457451</v>
+        <v>33486725</v>
       </c>
       <c r="E7" t="s">
         <v>34</v>
@@ -1432,7 +1421,7 @@
         <v>227463</v>
       </c>
       <c r="D8">
-        <v>228076</v>
+        <v>228289</v>
       </c>
       <c r="E8" t="s">
         <v>39</v>
@@ -1458,7 +1447,7 @@
         <v>348401</v>
       </c>
       <c r="D9">
-        <v>638780</v>
+        <v>639331</v>
       </c>
       <c r="E9" t="s">
         <v>43</v>
@@ -1484,19 +1473,19 @@
         <v>372919</v>
       </c>
       <c r="D10">
-        <v>1145303</v>
-      </c>
-      <c r="E10" t="s">
+        <v>1146269</v>
+      </c>
+      <c r="E10">
+        <v>88343033</v>
+      </c>
+      <c r="F10" t="s">
         <v>47</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>48</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>49</v>
-      </c>
-      <c r="H10" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1510,19 +1499,19 @@
         <v>454476</v>
       </c>
       <c r="D11">
-        <v>2369795</v>
+        <v>2371923</v>
       </c>
       <c r="E11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" t="s">
         <v>51</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>52</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>53</v>
-      </c>
-      <c r="H11" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1536,24 +1525,24 @@
         <v>252251</v>
       </c>
       <c r="D12">
-        <v>2620541</v>
+        <v>2622784</v>
       </c>
       <c r="E12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" t="s">
         <v>55</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>56</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>57</v>
-      </c>
-      <c r="H12" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B13" t="s">
         <v>13</v>
@@ -1562,24 +1551,24 @@
         <v>203143</v>
       </c>
       <c r="D13">
-        <v>203645</v>
+        <v>203777</v>
       </c>
       <c r="E13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F13" t="s">
+        <v>51</v>
+      </c>
+      <c r="G13" t="s">
         <v>60</v>
       </c>
-      <c r="F13" t="s">
+      <c r="H13" t="s">
         <v>61</v>
-      </c>
-      <c r="G13" t="s">
-        <v>62</v>
-      </c>
-      <c r="H13" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B14" t="s">
         <v>18</v>
@@ -1588,24 +1577,24 @@
         <v>273461</v>
       </c>
       <c r="D14">
-        <v>472943</v>
+        <v>473283</v>
       </c>
       <c r="E14" t="s">
+        <v>62</v>
+      </c>
+      <c r="F14" t="s">
+        <v>63</v>
+      </c>
+      <c r="G14" t="s">
         <v>64</v>
       </c>
-      <c r="F14" t="s">
+      <c r="H14" t="s">
         <v>65</v>
-      </c>
-      <c r="G14" t="s">
-        <v>66</v>
-      </c>
-      <c r="H14" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B15" t="s">
         <v>23</v>
@@ -1614,24 +1603,24 @@
         <v>237115</v>
       </c>
       <c r="D15">
-        <v>658439</v>
+        <v>658971</v>
       </c>
       <c r="E15" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" t="s">
+        <v>67</v>
+      </c>
+      <c r="G15" t="s">
         <v>68</v>
       </c>
-      <c r="F15" t="s">
+      <c r="H15" t="s">
         <v>69</v>
-      </c>
-      <c r="G15" t="s">
-        <v>70</v>
-      </c>
-      <c r="H15" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B16" t="s">
         <v>28</v>
@@ -1640,24 +1629,24 @@
         <v>199739</v>
       </c>
       <c r="D16">
-        <v>900123</v>
+        <v>900882</v>
       </c>
       <c r="E16" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" t="s">
+        <v>71</v>
+      </c>
+      <c r="G16" t="s">
         <v>72</v>
       </c>
-      <c r="F16" t="s">
+      <c r="H16" t="s">
         <v>73</v>
-      </c>
-      <c r="G16" t="s">
-        <v>74</v>
-      </c>
-      <c r="H16" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B17" t="s">
         <v>33</v>
@@ -1666,24 +1655,24 @@
         <v>58228</v>
       </c>
       <c r="D17">
-        <v>505729</v>
+        <v>506050</v>
       </c>
       <c r="E17" t="s">
+        <v>74</v>
+      </c>
+      <c r="F17" t="s">
+        <v>75</v>
+      </c>
+      <c r="G17" t="s">
         <v>76</v>
       </c>
-      <c r="F17" t="s">
+      <c r="H17" t="s">
         <v>77</v>
-      </c>
-      <c r="G17" t="s">
-        <v>78</v>
-      </c>
-      <c r="H17" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B18" t="s">
         <v>13</v>
@@ -1692,24 +1681,24 @@
         <v>578178</v>
       </c>
       <c r="D18">
-        <v>579295</v>
+        <v>579612</v>
       </c>
       <c r="E18" t="s">
+        <v>79</v>
+      </c>
+      <c r="F18" t="s">
+        <v>80</v>
+      </c>
+      <c r="G18" t="s">
         <v>81</v>
       </c>
-      <c r="F18" t="s">
+      <c r="H18" t="s">
         <v>82</v>
-      </c>
-      <c r="G18" t="s">
-        <v>83</v>
-      </c>
-      <c r="H18" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B19" t="s">
         <v>18</v>
@@ -1718,24 +1707,24 @@
         <v>600129</v>
       </c>
       <c r="D19">
-        <v>891908</v>
+        <v>892542</v>
       </c>
       <c r="E19" t="s">
+        <v>83</v>
+      </c>
+      <c r="F19" t="s">
+        <v>84</v>
+      </c>
+      <c r="G19" t="s">
         <v>85</v>
       </c>
-      <c r="F19" t="s">
+      <c r="H19" t="s">
         <v>86</v>
-      </c>
-      <c r="G19" t="s">
-        <v>87</v>
-      </c>
-      <c r="H19" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B20" t="s">
         <v>23</v>
@@ -1744,24 +1733,24 @@
         <v>354255</v>
       </c>
       <c r="D20">
-        <v>768484</v>
+        <v>769084</v>
       </c>
       <c r="E20" t="s">
+        <v>87</v>
+      </c>
+      <c r="F20" t="s">
+        <v>88</v>
+      </c>
+      <c r="G20" t="s">
         <v>89</v>
       </c>
-      <c r="F20" t="s">
+      <c r="H20" t="s">
         <v>90</v>
-      </c>
-      <c r="G20" t="s">
-        <v>91</v>
-      </c>
-      <c r="H20" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B21" t="s">
         <v>28</v>
@@ -1770,24 +1759,24 @@
         <v>179252</v>
       </c>
       <c r="D21">
-        <v>596028</v>
+        <v>596490</v>
       </c>
       <c r="E21" t="s">
+        <v>91</v>
+      </c>
+      <c r="F21" t="s">
+        <v>92</v>
+      </c>
+      <c r="G21" t="s">
         <v>93</v>
       </c>
-      <c r="F21" t="s">
+      <c r="H21" t="s">
         <v>94</v>
-      </c>
-      <c r="G21" t="s">
-        <v>95</v>
-      </c>
-      <c r="H21" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B22" t="s">
         <v>33</v>
@@ -1796,146 +1785,146 @@
         <v>32971</v>
       </c>
       <c r="D22">
-        <v>223936</v>
+        <v>224040</v>
       </c>
       <c r="E22" t="s">
+        <v>95</v>
+      </c>
+      <c r="F22" t="s">
+        <v>96</v>
+      </c>
+      <c r="G22" t="s">
         <v>97</v>
       </c>
-      <c r="F22" t="s">
-        <v>98</v>
-      </c>
-      <c r="G22" t="s">
-        <v>99</v>
-      </c>
       <c r="H22" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B23" t="s">
         <v>13</v>
       </c>
       <c r="C23">
-        <v>71147</v>
+        <v>71612</v>
       </c>
       <c r="D23">
-        <v>71323</v>
+        <v>71849</v>
       </c>
       <c r="E23" t="s">
+        <v>99</v>
+      </c>
+      <c r="F23" t="s">
+        <v>100</v>
+      </c>
+      <c r="G23" t="s">
         <v>101</v>
       </c>
-      <c r="F23" t="s">
+      <c r="H23" t="s">
         <v>102</v>
-      </c>
-      <c r="G23" t="s">
-        <v>103</v>
-      </c>
-      <c r="H23" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B24" t="s">
         <v>18</v>
       </c>
       <c r="C24">
-        <v>53789</v>
+        <v>54125</v>
       </c>
       <c r="D24">
-        <v>61829</v>
+        <v>62238</v>
       </c>
       <c r="E24" t="s">
+        <v>103</v>
+      </c>
+      <c r="F24">
+        <v>79</v>
+      </c>
+      <c r="G24" t="s">
+        <v>104</v>
+      </c>
+      <c r="H24" t="s">
         <v>105</v>
-      </c>
-      <c r="F24" t="s">
-        <v>106</v>
-      </c>
-      <c r="G24" t="s">
-        <v>107</v>
-      </c>
-      <c r="H24" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B25" t="s">
         <v>23</v>
       </c>
       <c r="C25">
-        <v>20044</v>
+        <v>20155</v>
       </c>
       <c r="D25">
-        <v>24670</v>
+        <v>24806</v>
       </c>
       <c r="E25" t="s">
+        <v>106</v>
+      </c>
+      <c r="F25" t="s">
+        <v>107</v>
+      </c>
+      <c r="G25" t="s">
+        <v>108</v>
+      </c>
+      <c r="H25" t="s">
         <v>109</v>
-      </c>
-      <c r="F25" t="s">
-        <v>110</v>
-      </c>
-      <c r="G25" t="s">
-        <v>111</v>
-      </c>
-      <c r="H25" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B26" t="s">
         <v>28</v>
       </c>
       <c r="C26">
-        <v>5794</v>
+        <v>5818</v>
       </c>
       <c r="D26">
-        <v>7647</v>
+        <v>7682</v>
       </c>
       <c r="E26" t="s">
+        <v>110</v>
+      </c>
+      <c r="F26" t="s">
+        <v>111</v>
+      </c>
+      <c r="G26" t="s">
+        <v>112</v>
+      </c>
+      <c r="H26" t="s">
         <v>113</v>
-      </c>
-      <c r="F26" t="s">
-        <v>114</v>
-      </c>
-      <c r="G26" t="s">
-        <v>115</v>
-      </c>
-      <c r="H26" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B27" t="s">
         <v>33</v>
       </c>
       <c r="C27">
-        <v>852</v>
+        <v>854</v>
       </c>
       <c r="D27">
-        <v>1371</v>
+        <v>1373</v>
       </c>
       <c r="E27" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F27" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G27" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H27">
         <v>0</v>

</xml_diff>